<commit_message>
Leads: 2026-10-08 05:30 UTC (cycle 3)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-08.xlsx
+++ b/output/leads_2026-10-08.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -625,6 +625,62 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Minuteman Electric &amp; HVAC in Idaho Falls, ID - HVAC and Electrician</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>minutemanservicesid.com</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>https://minutemanservicesid.com/services/furnace-repair/</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>solutions@minutemanservicesid.com</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>(208) 520-7885</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Idaho Falls ID</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>90</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>furnace repair Idaho Falls ID</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-08 05:35 UTC (cycle 6)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-08.xlsx
+++ b/output/leads_2026-10-08.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -646,7 +646,6 @@
           <t>https://minutemanservicesid.com/services/furnace-repair/</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>solutions@minutemanservicesid.com</t>
@@ -676,6 +675,174 @@
         </is>
       </c>
       <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>DC Air Conditioning &amp; Heating</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>dcachvac.com</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>https://dcachvac.com/ac-repair-services-in-washington-dc/</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>accurate1634@gmail.com</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>(202) 985-8885</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Washington DC</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>100</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>air conditioning repair Washington DC</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>AC REPAIR DC</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>acrepairdc.com</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>https://acrepairdc.com/</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>rishu.animator@gmail.com</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>202-609-9803</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Washington DC</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>88</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>air conditioning repair Washington DC</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>L &amp; L Roofing Co. â Lincoln, Nebraska</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>llroof.com</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>http://www.llroof.com/</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>danlenz27@gmail.com</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>402-580-2032</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Lincoln NE</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>68</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>roofer Lincoln NE</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
         <is>
           <t>2026-10-08</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-08 05:44 UTC (cycle 12)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-08.xlsx
+++ b/output/leads_2026-10-08.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -701,7 +701,6 @@
           <t>https://dcachvac.com/ac-repair-services-in-washington-dc/</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>accurate1634@gmail.com</t>
@@ -757,7 +756,6 @@
           <t>https://acrepairdc.com/</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>rishu.animator@gmail.com</t>
@@ -813,7 +811,6 @@
           <t>http://www.llroof.com/</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>danlenz27@gmail.com</t>
@@ -843,6 +840,126 @@
         </is>
       </c>
       <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>FrontRunner</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>frontrunnerconstruction.com</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>https://www.frontrunnerconstruction.com/roof-replacement-york-pa</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>York County</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>frontrunnerconst@gmail.com</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>(717)-208-2202</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>York PA</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>90</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>roof replacement York PA</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Roofing York PA</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>roofingyorkpa.com</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>https://roofingyorkpa.com/</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>York County</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>admin@roofingyorkpa.com</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>(888) 217-3626</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>York PA</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>80</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>roof replacement York PA</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
         <is>
           <t>2026-10-08</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-08 06:56 UTC (cycle 62)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-08.xlsx
+++ b/output/leads_2026-10-08.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -965,6 +965,62 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Metal Roofing in Palm Bay, FL | 3LP Roofing Inc</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>3lproofing.com</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>https://www.3lproofing.com/metal-roofing-palm-bay-fl</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>office@3lproofing.com</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>(321) 326-0817</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Palm Bay FL</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>100</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Palm Bay FL</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-08 06:59 UTC (cycle 64)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-08.xlsx
+++ b/output/leads_2026-10-08.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -986,7 +986,6 @@
           <t>https://www.3lproofing.com/metal-roofing-palm-bay-fl</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
           <t>office@3lproofing.com</t>
@@ -1016,6 +1015,66 @@
         </is>
       </c>
       <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>The #1 Water, Fire Restoration, and Mold Remediation Service in Atlanta</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>airdropatlanta.com</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>https://www.airdropatlanta.com/emergency-plumber-atlanta/</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Sandy Springs</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>info@airdropatlanta.com</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>678-374-9247</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Atlanta GA</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>90</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>emergency plumber Atlanta GA</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
         <is>
           <t>2026-10-08</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-08 07:02 UTC (cycle 66)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-08.xlsx
+++ b/output/leads_2026-10-08.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1080,6 +1080,66 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>San Diego Turbo Drains</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>turbodrains.com</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>https://www.turbodrains.com/</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>San Diego</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>info@turbodrains.com</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>858-888-6788</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>San Diego CA</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>90</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>drain cleaning service San Diego CA</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-08 07:05 UTC (cycle 68)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-08.xlsx
+++ b/output/leads_2026-10-08.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1140,6 +1140,66 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Furnace Repair Colorado Springs</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>furnacerepaircoloradosprings.com</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>https://www.furnacerepaircoloradosprings.com/</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Colorado Springs</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>info@furnacerepaircoloradosprings.com</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>719-602-8787</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Colorado Springs CO</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>90</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>furnace repair Colorado Springs CO</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-08 07:07 UTC (cycle 69)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-08.xlsx
+++ b/output/leads_2026-10-08.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1200,6 +1200,66 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>AT Plumbing Services</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>atplumbingservices.com</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>https://www.atplumbingservices.com/portland-maine</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Plumbing Services</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>a.tplumbing207@gmail.com</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>(207)-707-3170</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Portland ME</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>90</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>plumbing company Portland ME</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-08 07:09 UTC (cycle 70)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-08.xlsx
+++ b/output/leads_2026-10-08.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:L17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1260,6 +1260,186 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>First Call Air Conditioning &amp; Heating Repair</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>firstcallairconditioning.com</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>https://firstcallairconditioning.com/locations/utica-ny.html</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Often How</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>dispatch@firstcallairconditioning.com</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>(329) 202-9924</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Utica NY</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>90</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>air conditioning repair Utica NY</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Plumbing Services | Brooks Plumbing | Garland &amp; Dallas</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>brooksplumbingtexas.com</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>https://www.brooksplumbingtexas.com/</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Brooks Plumbing</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>info@brooksplumbingtexas.com</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>(214) 368-3838</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Garland TX</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>90</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>plumbing company Garland TX</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Halo Roofing</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>haloroofingomaha.com</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>https://www.haloroofingomaha.com/services/metal-roofing-company/</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Halo Roofing</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>john@smith.com</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>(402) 599-3526</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Omaha NE</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>90</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Omaha NE</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-08 07:15 UTC (cycle 74)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-08.xlsx
+++ b/output/leads_2026-10-08.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L17"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1440,6 +1440,66 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Dream Craft Builders</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>dreamcraftbuildersde.com</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>https://dreamcraftbuildersde.com/services/roofing/dover-de</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Kent County</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>dreamcraftbuildersconstruction@gmail.com</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>302-444-1006</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Dover DE</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>90</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>roof replacement Dover DE</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-08 07:23 UTC (cycle 79)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-08.xlsx
+++ b/output/leads_2026-10-08.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L18"/>
+  <dimension ref="A1:L19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1500,6 +1500,66 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>www.zoplumbing.com</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>zoplumbing.com</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>https://www.zoplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Serving Maryland</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>info@zoplumbing.com</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>(301) 401-1181</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Frederick MD</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>90</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>drain cleaning service Frederick MD</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-08 07:24 UTC (cycle 80)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-08.xlsx
+++ b/output/leads_2026-10-08.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L19"/>
+  <dimension ref="A1:L20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1560,6 +1560,66 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>HVAC New Braunfels TX | AC Repair &amp; Installation | Amazing Air Solutions</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>amazingairsolutions.co</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>https://amazingairsolutions.co/service-area/new-braunfels</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>China Grove</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>amazingairsolutions@gmail.com</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>(210) 390-1925</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>New Braunfels TX</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>84</v>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>HVAC contractor New Braunfels TX</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-08 07:29 UTC (cycle 83)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-08.xlsx
+++ b/output/leads_2026-10-08.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L20"/>
+  <dimension ref="A1:L21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1620,6 +1620,62 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Five Star Plumbing</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>fivestarplumbingservices.com</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>https://www.fivestarplumbingservices.com/plumbing-services-dayton-oh/</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>service@fivestarplumbingservices.com</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>(937) 902-6195</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Dayton OH</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>100</v>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>plumbing company Dayton OH</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-08 07:30 UTC (cycle 84)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-08.xlsx
+++ b/output/leads_2026-10-08.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L21"/>
+  <dimension ref="A1:L22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1641,7 +1641,6 @@
           <t>https://www.fivestarplumbingservices.com/plumbing-services-dayton-oh/</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
           <t>service@fivestarplumbingservices.com</t>
@@ -1671,6 +1670,66 @@
         </is>
       </c>
       <c r="L21" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>RSJ Mechanical</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>rsjmechanical.com</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>https://www.rsjmechanical.com/idaho-falls/</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Idaho Falls</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>rsjmechanical@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>(208) 521-3764</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Idaho Falls ID</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>90</v>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>heating and cooling company Idaho Falls ID</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
         <is>
           <t>2026-10-08</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-08 15:27 UTC (cycle 1)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-08.xlsx
+++ b/output/leads_2026-10-08.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L22"/>
+  <dimension ref="A1:L23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1735,6 +1735,66 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Roofing Company in Fayetteville, AR | Repair and Replacement</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>fayettevilleroofpros.com</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>https://fayettevilleroofpros.com/</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Questions Fayetteville</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>hello@fayettevilleroofpros.com</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>(479) 480-5320</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Fayetteville AR</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>90</v>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>roof repair company Fayetteville AR</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-08 15:28 UTC (cycle 2)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-08.xlsx
+++ b/output/leads_2026-10-08.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L23"/>
+  <dimension ref="A1:L24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1795,6 +1795,66 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Mahalo Mechanical</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>mahalomechanical.com</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>https://mahalomechanical.com/ac-installation/</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Mahalo Mechanical</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>mahalomechanical@gmail.com</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>(757)-335-9628</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Virginia Beach VA</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>90</v>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>AC installation Virginia Beach VA</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-08 15:31 UTC (cycle 4)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-08.xlsx
+++ b/output/leads_2026-10-08.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L24"/>
+  <dimension ref="A1:L25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1855,6 +1855,62 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Pulles Plumbing</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>pullesplumbing.com</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>https://pullesplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>cpulles@bellsouth.net</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>305 558 0410</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Miami FL</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>90</v>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>plumbing company Miami FL</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-08 15:33 UTC (cycle 5)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-08.xlsx
+++ b/output/leads_2026-10-08.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L25"/>
+  <dimension ref="A1:L26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1876,7 +1876,6 @@
           <t>https://pullesplumbing.com/</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
         <is>
           <t>cpulles@bellsouth.net</t>
@@ -1906,6 +1905,66 @@
         </is>
       </c>
       <c r="L25" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Plumber Services | Wickey Plumbing LLC | Fort Wayne, IN</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>wickeyplumbing.com</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>https://www.wickeyplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Learn More</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>wickeyplumbing@gmail.com</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>(260) 409-5128</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Fort Wayne IN</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>100</v>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>plumbing company Fort Wayne IN</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
         <is>
           <t>2026-10-08</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-08 15:36 UTC (cycle 7)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-08.xlsx
+++ b/output/leads_2026-10-08.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L26"/>
+  <dimension ref="A1:L27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1970,6 +1970,66 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Yates Roofing &amp; Construction LLC</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>yatesok.com</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>https://www.yatesok.com/</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Why Oklahoma</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>service@yatesok.com</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>405-607-0966</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Oklahoma City OK</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>90</v>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>roof repair company Oklahoma City OK</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-08 15:37 UTC (cycle 8)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-08.xlsx
+++ b/output/leads_2026-10-08.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L27"/>
+  <dimension ref="A1:L30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2030,6 +2030,182 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Luke Lays Pipe</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>lukelayspipe.com</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>https://lukelayspipe.com/services/sewer-line-repair/</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>info@lukelayspipe.com</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>(734) 748-4831</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Nashville TN</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>90</v>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>sewer repair Nashville TN</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Astoria Plumbing &amp; Water Heater Specialist</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>plumberqueensny.us</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>https://plumberqueensny.us/</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Your Most</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>info@plumberqueensny.us</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>929-244-0432</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Queens NY</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
+        <v>90</v>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>emergency plumber Queens NY</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>JC Heating &amp; Air LLC</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>jcheatingandairllc.com</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>https://www.jcheatingandairllc.com/</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Middle Tennessee</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>company37064@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>(615) 524-9575</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Franklin TN</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
+        <v>86</v>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>heating and cooling company Franklin TN</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-08 21:17 UTC (cycle 5)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-08.xlsx
+++ b/output/leads_2026-10-08.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L30"/>
+  <dimension ref="A1:L31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2051,7 +2051,6 @@
           <t>https://lukelayspipe.com/services/sewer-line-repair/</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
           <t>info@lukelayspipe.com</t>
@@ -2201,6 +2200,66 @@
         </is>
       </c>
       <c r="L30" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Roofing Company in Bellevue, WA | Integrity Roofing Services LLC</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>integrityroofingservicesllc.com</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>https://integrityroofingservicesllc.com/locations/roofing-company-bellevue-wa</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Roofing Company</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>contact@integrityroofingservicesllc.com</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>(253) 468-8994</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Bellevue WA</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
+        <v>90</v>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>residential roofing company Bellevue WA</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
         <is>
           <t>2026-10-08</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-08 21:28 UTC (cycle 12)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-08.xlsx
+++ b/output/leads_2026-10-08.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L31"/>
+  <dimension ref="A1:L32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2265,6 +2265,66 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>plumbingbismarck.com</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>plumbingbismarck.com</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>https://plumbingbismarck.com/</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Toilet Humming</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>abdullah0razzaq@gmail.com</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>(701) 937-3701</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Bismarck ND</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
+        <v>90</v>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>emergency plumber Bismarck ND</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>